<commit_message>
Full dashboard with scrollable replenishment view, search, and WH SOH column
</commit_message>
<xml_diff>
--- a/Reports/Auto_Replenishment_Action_Plan.xlsx
+++ b/Reports/Auto_Replenishment_Action_Plan.xlsx
@@ -8053,7 +8053,7 @@
         <v>1.87</v>
       </c>
       <c r="J2">
-        <v>-752</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1457</v>
@@ -8091,7 +8091,7 @@
         <v>0.1</v>
       </c>
       <c r="J3">
-        <v>-150</v>
+        <v>0</v>
       </c>
       <c r="K3">
         <v>17</v>
@@ -8129,7 +8129,7 @@
         <v>0.17</v>
       </c>
       <c r="J4">
-        <v>-150</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <v>29</v>
@@ -8167,7 +8167,7 @@
         <v>0.13</v>
       </c>
       <c r="J5">
-        <v>-135</v>
+        <v>0</v>
       </c>
       <c r="K5">
         <v>16</v>
@@ -8205,7 +8205,7 @@
         <v>0.17</v>
       </c>
       <c r="J6">
-        <v>-126</v>
+        <v>0</v>
       </c>
       <c r="K6">
         <v>22</v>
@@ -8243,7 +8243,7 @@
         <v>0.1</v>
       </c>
       <c r="J7">
-        <v>-120</v>
+        <v>0</v>
       </c>
       <c r="K7">
         <v>14</v>
@@ -8281,7 +8281,7 @@
         <v>0.13</v>
       </c>
       <c r="J8">
-        <v>-112</v>
+        <v>0</v>
       </c>
       <c r="K8">
         <v>18</v>
@@ -8319,7 +8319,7 @@
         <v>0.13</v>
       </c>
       <c r="J9">
-        <v>-112</v>
+        <v>0</v>
       </c>
       <c r="K9">
         <v>8</v>
@@ -8357,7 +8357,7 @@
         <v>0.23</v>
       </c>
       <c r="J10">
-        <v>-111</v>
+        <v>0</v>
       </c>
       <c r="K10">
         <v>16</v>
@@ -8395,7 +8395,7 @@
         <v>0.1</v>
       </c>
       <c r="J11">
-        <v>-110</v>
+        <v>0</v>
       </c>
       <c r="K11">
         <v>13</v>
@@ -8433,7 +8433,7 @@
         <v>0.23</v>
       </c>
       <c r="J12">
-        <v>-107</v>
+        <v>0</v>
       </c>
       <c r="K12">
         <v>31</v>
@@ -8471,7 +8471,7 @@
         <v>0.1</v>
       </c>
       <c r="J13">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="K13">
         <v>12</v>
@@ -8509,7 +8509,7 @@
         <v>0.1</v>
       </c>
       <c r="J14">
-        <v>-100</v>
+        <v>0</v>
       </c>
       <c r="K14">
         <v>12</v>
@@ -8547,7 +8547,7 @@
         <v>0.17</v>
       </c>
       <c r="J15">
-        <v>-90</v>
+        <v>0</v>
       </c>
       <c r="K15">
         <v>8</v>
@@ -8585,7 +8585,7 @@
         <v>0.1</v>
       </c>
       <c r="J16">
-        <v>-90</v>
+        <v>0</v>
       </c>
       <c r="K16">
         <v>11</v>
@@ -8623,7 +8623,7 @@
         <v>0.1</v>
       </c>
       <c r="J17">
-        <v>-80</v>
+        <v>0</v>
       </c>
       <c r="K17">
         <v>10</v>
@@ -8661,7 +8661,7 @@
         <v>0.1</v>
       </c>
       <c r="J18">
-        <v>-80</v>
+        <v>0</v>
       </c>
       <c r="K18">
         <v>10</v>
@@ -8699,7 +8699,7 @@
         <v>0.13</v>
       </c>
       <c r="J19">
-        <v>-75</v>
+        <v>0</v>
       </c>
       <c r="K19">
         <v>13</v>
@@ -8737,7 +8737,7 @@
         <v>0.1</v>
       </c>
       <c r="J20">
-        <v>-70</v>
+        <v>0</v>
       </c>
       <c r="K20">
         <v>10</v>
@@ -8775,7 +8775,7 @@
         <v>0.2</v>
       </c>
       <c r="J21">
-        <v>-70</v>
+        <v>0</v>
       </c>
       <c r="K21">
         <v>19</v>
@@ -8813,7 +8813,7 @@
         <v>0.1</v>
       </c>
       <c r="J22">
-        <v>-70</v>
+        <v>0</v>
       </c>
       <c r="K22">
         <v>10</v>
@@ -8851,7 +8851,7 @@
         <v>0.1</v>
       </c>
       <c r="J23">
-        <v>-70</v>
+        <v>0</v>
       </c>
       <c r="K23">
         <v>10</v>
@@ -8889,7 +8889,7 @@
         <v>0.1</v>
       </c>
       <c r="J24">
-        <v>-70</v>
+        <v>0</v>
       </c>
       <c r="K24">
         <v>10</v>
@@ -8927,7 +8927,7 @@
         <v>2.47</v>
       </c>
       <c r="J25">
-        <v>-68</v>
+        <v>0</v>
       </c>
       <c r="K25">
         <v>239</v>
@@ -8965,7 +8965,7 @@
         <v>0.17</v>
       </c>
       <c r="J26">
-        <v>-66</v>
+        <v>0</v>
       </c>
       <c r="K26">
         <v>15</v>
@@ -9003,7 +9003,7 @@
         <v>0.17</v>
       </c>
       <c r="J27">
-        <v>-66</v>
+        <v>0</v>
       </c>
       <c r="K27">
         <v>12</v>
@@ -9041,7 +9041,7 @@
         <v>0.17</v>
       </c>
       <c r="J28">
-        <v>-66</v>
+        <v>0</v>
       </c>
       <c r="K28">
         <v>15</v>
@@ -9079,7 +9079,7 @@
         <v>0.17</v>
       </c>
       <c r="J29">
-        <v>-66</v>
+        <v>0</v>
       </c>
       <c r="K29">
         <v>13</v>
@@ -9117,7 +9117,7 @@
         <v>0.23</v>
       </c>
       <c r="J30">
-        <v>-64</v>
+        <v>0</v>
       </c>
       <c r="K30">
         <v>21</v>
@@ -9155,7 +9155,7 @@
         <v>0.17</v>
       </c>
       <c r="J31">
-        <v>-60</v>
+        <v>0</v>
       </c>
       <c r="K31">
         <v>14</v>
@@ -9193,7 +9193,7 @@
         <v>0.6</v>
       </c>
       <c r="J32">
-        <v>-60</v>
+        <v>0</v>
       </c>
       <c r="K32">
         <v>52</v>
@@ -9231,7 +9231,7 @@
         <v>0.1</v>
       </c>
       <c r="J33">
-        <v>-60</v>
+        <v>0</v>
       </c>
       <c r="K33">
         <v>10</v>
@@ -9269,7 +9269,7 @@
         <v>0.63</v>
       </c>
       <c r="J34">
-        <v>-60</v>
+        <v>0</v>
       </c>
       <c r="K34">
         <v>14</v>
@@ -9307,7 +9307,7 @@
         <v>0.1</v>
       </c>
       <c r="J35">
-        <v>-60</v>
+        <v>0</v>
       </c>
       <c r="K35">
         <v>10</v>
@@ -9345,7 +9345,7 @@
         <v>0.13</v>
       </c>
       <c r="J36">
-        <v>-60</v>
+        <v>0</v>
       </c>
       <c r="K36">
         <v>11</v>
@@ -9383,7 +9383,7 @@
         <v>0.1</v>
       </c>
       <c r="J37">
-        <v>-60</v>
+        <v>0</v>
       </c>
       <c r="K37">
         <v>10</v>
@@ -9421,7 +9421,7 @@
         <v>0.13</v>
       </c>
       <c r="J38">
-        <v>-60</v>
+        <v>0</v>
       </c>
       <c r="K38">
         <v>11</v>
@@ -9459,7 +9459,7 @@
         <v>0.43</v>
       </c>
       <c r="J39">
-        <v>-57</v>
+        <v>0</v>
       </c>
       <c r="K39">
         <v>12</v>
@@ -9497,7 +9497,7 @@
         <v>0.37</v>
       </c>
       <c r="J40">
-        <v>-54</v>
+        <v>0</v>
       </c>
       <c r="K40">
         <v>30</v>
@@ -9535,7 +9535,7 @@
         <v>0.17</v>
       </c>
       <c r="J41">
-        <v>-54</v>
+        <v>0</v>
       </c>
       <c r="K41">
         <v>10</v>
@@ -9573,7 +9573,7 @@
         <v>0.47</v>
       </c>
       <c r="J42">
-        <v>-53</v>
+        <v>0</v>
       </c>
       <c r="K42">
         <v>38</v>
@@ -9611,7 +9611,7 @@
         <v>0.13</v>
       </c>
       <c r="J43">
-        <v>-52</v>
+        <v>0</v>
       </c>
       <c r="K43">
         <v>10</v>
@@ -9649,7 +9649,7 @@
         <v>0.1</v>
       </c>
       <c r="J44">
-        <v>-50</v>
+        <v>0</v>
       </c>
       <c r="K44">
         <v>10</v>
@@ -9687,7 +9687,7 @@
         <v>0.1</v>
       </c>
       <c r="J45">
-        <v>-50</v>
+        <v>0</v>
       </c>
       <c r="K45">
         <v>10</v>
@@ -9725,7 +9725,7 @@
         <v>0.27</v>
       </c>
       <c r="J46">
-        <v>-48</v>
+        <v>0</v>
       </c>
       <c r="K46">
         <v>20</v>
@@ -9763,7 +9763,7 @@
         <v>0.17</v>
       </c>
       <c r="J47">
-        <v>-48</v>
+        <v>0</v>
       </c>
       <c r="K47">
         <v>9</v>
@@ -9801,7 +9801,7 @@
         <v>0.13</v>
       </c>
       <c r="J48">
-        <v>-45</v>
+        <v>0</v>
       </c>
       <c r="K48">
         <v>10</v>
@@ -9839,7 +9839,7 @@
         <v>0.2</v>
       </c>
       <c r="J49">
-        <v>-45</v>
+        <v>0</v>
       </c>
       <c r="K49">
         <v>8</v>
@@ -9877,7 +9877,7 @@
         <v>0.13</v>
       </c>
       <c r="J50">
-        <v>-45</v>
+        <v>0</v>
       </c>
       <c r="K50">
         <v>10</v>
@@ -9915,7 +9915,7 @@
         <v>0.37</v>
       </c>
       <c r="J51">
-        <v>-43</v>
+        <v>0</v>
       </c>
       <c r="K51">
         <v>26</v>
@@ -9953,7 +9953,7 @@
         <v>0.23</v>
       </c>
       <c r="J52">
-        <v>-42</v>
+        <v>0</v>
       </c>
       <c r="K52">
         <v>8</v>
@@ -9991,7 +9991,7 @@
         <v>0.23</v>
       </c>
       <c r="J53">
-        <v>-42</v>
+        <v>0</v>
       </c>
       <c r="K53">
         <v>15</v>
@@ -10029,7 +10029,7 @@
         <v>0.17</v>
       </c>
       <c r="J54">
-        <v>-42</v>
+        <v>0</v>
       </c>
       <c r="K54">
         <v>8</v>
@@ -10067,7 +10067,7 @@
         <v>0.1</v>
       </c>
       <c r="J55">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="K55">
         <v>10</v>
@@ -10105,7 +10105,7 @@
         <v>0.1</v>
       </c>
       <c r="J56">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="K56">
         <v>10</v>
@@ -10143,7 +10143,7 @@
         <v>0.1</v>
       </c>
       <c r="J57">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="K57">
         <v>10</v>
@@ -10181,7 +10181,7 @@
         <v>0.1</v>
       </c>
       <c r="J58">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="K58">
         <v>10</v>
@@ -10219,7 +10219,7 @@
         <v>0.1</v>
       </c>
       <c r="J59">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="K59">
         <v>10</v>
@@ -10257,7 +10257,7 @@
         <v>0.2</v>
       </c>
       <c r="J60">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="K60">
         <v>13</v>
@@ -10295,7 +10295,7 @@
         <v>0.1</v>
       </c>
       <c r="J61">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="K61">
         <v>10</v>
@@ -10333,7 +10333,7 @@
         <v>0.1</v>
       </c>
       <c r="J62">
-        <v>-40</v>
+        <v>0</v>
       </c>
       <c r="K62">
         <v>10</v>
@@ -10371,7 +10371,7 @@
         <v>0.33</v>
       </c>
       <c r="J63">
-        <v>-39</v>
+        <v>0</v>
       </c>
       <c r="K63">
         <v>22</v>
@@ -10409,7 +10409,7 @@
         <v>0.23</v>
       </c>
       <c r="J64">
-        <v>-38</v>
+        <v>0</v>
       </c>
       <c r="K64">
         <v>15</v>
@@ -10447,7 +10447,7 @@
         <v>0.23</v>
       </c>
       <c r="J65">
-        <v>-38</v>
+        <v>0</v>
       </c>
       <c r="K65">
         <v>8</v>
@@ -10485,7 +10485,7 @@
         <v>0.13</v>
       </c>
       <c r="J66">
-        <v>-37</v>
+        <v>0</v>
       </c>
       <c r="K66">
         <v>8</v>
@@ -10523,7 +10523,7 @@
         <v>0.13</v>
       </c>
       <c r="J67">
-        <v>-37</v>
+        <v>0</v>
       </c>
       <c r="K67">
         <v>10</v>
@@ -10561,7 +10561,7 @@
         <v>0.13</v>
       </c>
       <c r="J68">
-        <v>-37</v>
+        <v>0</v>
       </c>
       <c r="K68">
         <v>10</v>
@@ -10599,7 +10599,7 @@
         <v>1.93</v>
       </c>
       <c r="J69">
-        <v>-36</v>
+        <v>0</v>
       </c>
       <c r="K69">
         <v>124</v>
@@ -10637,7 +10637,7 @@
         <v>0.17</v>
       </c>
       <c r="J70">
-        <v>-36</v>
+        <v>0</v>
       </c>
       <c r="K70">
         <v>10</v>
@@ -10675,7 +10675,7 @@
         <v>0.23</v>
       </c>
       <c r="J71">
-        <v>-34</v>
+        <v>0</v>
       </c>
       <c r="K71">
         <v>14</v>
@@ -10713,7 +10713,7 @@
         <v>0.27</v>
       </c>
       <c r="J72">
-        <v>-33</v>
+        <v>0</v>
       </c>
       <c r="K72">
         <v>16</v>
@@ -10751,7 +10751,7 @@
         <v>0.2</v>
       </c>
       <c r="J73">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K73">
         <v>11</v>
@@ -10789,7 +10789,7 @@
         <v>0.33</v>
       </c>
       <c r="J74">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K74">
         <v>19</v>
@@ -10827,7 +10827,7 @@
         <v>0.1</v>
       </c>
       <c r="J75">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K75">
         <v>10</v>
@@ -10865,7 +10865,7 @@
         <v>0.1</v>
       </c>
       <c r="J76">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K76">
         <v>10</v>
@@ -10903,7 +10903,7 @@
         <v>0.17</v>
       </c>
       <c r="J77">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K77">
         <v>10</v>
@@ -10941,7 +10941,7 @@
         <v>0.1</v>
       </c>
       <c r="J78">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K78">
         <v>10</v>
@@ -10979,7 +10979,7 @@
         <v>0.13</v>
       </c>
       <c r="J79">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K79">
         <v>10</v>
@@ -11017,7 +11017,7 @@
         <v>0.17</v>
       </c>
       <c r="J80">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K80">
         <v>10</v>
@@ -11055,7 +11055,7 @@
         <v>0.5</v>
       </c>
       <c r="J81">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K81">
         <v>16</v>
@@ -11093,7 +11093,7 @@
         <v>0.23</v>
       </c>
       <c r="J82">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K82">
         <v>13</v>
@@ -11131,7 +11131,7 @@
         <v>0.33</v>
       </c>
       <c r="J83">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K83">
         <v>19</v>
@@ -11169,7 +11169,7 @@
         <v>0.17</v>
       </c>
       <c r="J84">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K84">
         <v>10</v>
@@ -11207,7 +11207,7 @@
         <v>0.53</v>
       </c>
       <c r="J85">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K85">
         <v>18</v>
@@ -11245,7 +11245,7 @@
         <v>0.1</v>
       </c>
       <c r="J86">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K86">
         <v>8</v>
@@ -11283,7 +11283,7 @@
         <v>0.2</v>
       </c>
       <c r="J87">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K87">
         <v>11</v>
@@ -11321,7 +11321,7 @@
         <v>0.1</v>
       </c>
       <c r="J88">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K88">
         <v>10</v>
@@ -11359,7 +11359,7 @@
         <v>0.17</v>
       </c>
       <c r="J89">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K89">
         <v>10</v>
@@ -11397,7 +11397,7 @@
         <v>0.4</v>
       </c>
       <c r="J90">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K90">
         <v>23</v>
@@ -11435,7 +11435,7 @@
         <v>0.3</v>
       </c>
       <c r="J91">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K91">
         <v>17</v>
@@ -11473,7 +11473,7 @@
         <v>0.33</v>
       </c>
       <c r="J92">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K92">
         <v>19</v>
@@ -11511,7 +11511,7 @@
         <v>0.1</v>
       </c>
       <c r="J93">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K93">
         <v>10</v>
@@ -11549,7 +11549,7 @@
         <v>0.17</v>
       </c>
       <c r="J94">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K94">
         <v>10</v>
@@ -11587,7 +11587,7 @@
         <v>0.3</v>
       </c>
       <c r="J95">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K95">
         <v>15</v>
@@ -11625,7 +11625,7 @@
         <v>0.1</v>
       </c>
       <c r="J96">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K96">
         <v>10</v>
@@ -11663,7 +11663,7 @@
         <v>0.13</v>
       </c>
       <c r="J97">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K97">
         <v>10</v>
@@ -11701,7 +11701,7 @@
         <v>0.23</v>
       </c>
       <c r="J98">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K98">
         <v>13</v>
@@ -11739,7 +11739,7 @@
         <v>0.1</v>
       </c>
       <c r="J99">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K99">
         <v>10</v>
@@ -11777,7 +11777,7 @@
         <v>0.13</v>
       </c>
       <c r="J100">
-        <v>-30</v>
+        <v>0</v>
       </c>
       <c r="K100">
         <v>10</v>
@@ -11815,7 +11815,7 @@
         <v>0.77</v>
       </c>
       <c r="J101">
-        <v>-28</v>
+        <v>0</v>
       </c>
       <c r="K101">
         <v>43</v>
@@ -11853,7 +11853,7 @@
         <v>0.27</v>
       </c>
       <c r="J102">
-        <v>-26</v>
+        <v>0</v>
       </c>
       <c r="K102">
         <v>9</v>
@@ -11891,7 +11891,7 @@
         <v>0.23</v>
       </c>
       <c r="J103">
-        <v>-25</v>
+        <v>0</v>
       </c>
       <c r="K103">
         <v>12</v>
@@ -11929,7 +11929,7 @@
         <v>0.23</v>
       </c>
       <c r="J104">
-        <v>-25</v>
+        <v>0</v>
       </c>
       <c r="K104">
         <v>12</v>
@@ -11967,7 +11967,7 @@
         <v>0.2</v>
       </c>
       <c r="J105">
-        <v>-25</v>
+        <v>0</v>
       </c>
       <c r="K105">
         <v>10</v>
@@ -12005,7 +12005,7 @@
         <v>0.53</v>
       </c>
       <c r="J106">
-        <v>-24</v>
+        <v>0</v>
       </c>
       <c r="K106">
         <v>16</v>
@@ -12043,7 +12043,7 @@
         <v>0.67</v>
       </c>
       <c r="J107">
-        <v>-24</v>
+        <v>0</v>
       </c>
       <c r="K107">
         <v>34</v>
@@ -12081,7 +12081,7 @@
         <v>0.17</v>
       </c>
       <c r="J108">
-        <v>-24</v>
+        <v>0</v>
       </c>
       <c r="K108">
         <v>10</v>
@@ -12119,7 +12119,7 @@
         <v>0.17</v>
       </c>
       <c r="J109">
-        <v>-24</v>
+        <v>0</v>
       </c>
       <c r="K109">
         <v>10</v>
@@ -12157,7 +12157,7 @@
         <v>0.3</v>
       </c>
       <c r="J110">
-        <v>-23</v>
+        <v>0</v>
       </c>
       <c r="K110">
         <v>15</v>
@@ -12195,7 +12195,7 @@
         <v>0.13</v>
       </c>
       <c r="J111">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K111">
         <v>10</v>
@@ -12233,7 +12233,7 @@
         <v>0.27</v>
       </c>
       <c r="J112">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K112">
         <v>9</v>
@@ -12271,7 +12271,7 @@
         <v>0.13</v>
       </c>
       <c r="J113">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K113">
         <v>10</v>
@@ -12309,7 +12309,7 @@
         <v>0.4</v>
       </c>
       <c r="J114">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K114">
         <v>20</v>
@@ -12347,7 +12347,7 @@
         <v>0.13</v>
       </c>
       <c r="J115">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K115">
         <v>10</v>
@@ -12385,7 +12385,7 @@
         <v>0.13</v>
       </c>
       <c r="J116">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K116">
         <v>10</v>
@@ -12423,7 +12423,7 @@
         <v>0.13</v>
       </c>
       <c r="J117">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K117">
         <v>10</v>
@@ -12461,7 +12461,7 @@
         <v>0.13</v>
       </c>
       <c r="J118">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K118">
         <v>10</v>
@@ -12499,7 +12499,7 @@
         <v>0.4</v>
       </c>
       <c r="J119">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K119">
         <v>20</v>
@@ -12537,7 +12537,7 @@
         <v>0.13</v>
       </c>
       <c r="J120">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K120">
         <v>10</v>
@@ -12575,7 +12575,7 @@
         <v>0.13</v>
       </c>
       <c r="J121">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K121">
         <v>10</v>
@@ -12613,7 +12613,7 @@
         <v>0.13</v>
       </c>
       <c r="J122">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K122">
         <v>10</v>
@@ -12651,7 +12651,7 @@
         <v>0.5</v>
       </c>
       <c r="J123">
-        <v>-22</v>
+        <v>0</v>
       </c>
       <c r="K123">
         <v>25</v>
@@ -12689,7 +12689,7 @@
         <v>0.37</v>
       </c>
       <c r="J124">
-        <v>-21</v>
+        <v>0</v>
       </c>
       <c r="K124">
         <v>15</v>
@@ -12727,7 +12727,7 @@
         <v>0.47</v>
       </c>
       <c r="J125">
-        <v>-21</v>
+        <v>0</v>
       </c>
       <c r="K125">
         <v>15</v>
@@ -12765,7 +12765,7 @@
         <v>0.57</v>
       </c>
       <c r="J126">
-        <v>-21</v>
+        <v>0</v>
       </c>
       <c r="K126">
         <v>8</v>
@@ -12803,7 +12803,7 @@
         <v>0.33</v>
       </c>
       <c r="J127">
-        <v>-21</v>
+        <v>0</v>
       </c>
       <c r="K127">
         <v>16</v>
@@ -12841,7 +12841,7 @@
         <v>0.1</v>
       </c>
       <c r="J128">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K128">
         <v>10</v>
@@ -12879,7 +12879,7 @@
         <v>0.2</v>
       </c>
       <c r="J129">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K129">
         <v>10</v>
@@ -12917,7 +12917,7 @@
         <v>0.1</v>
       </c>
       <c r="J130">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K130">
         <v>10</v>
@@ -12955,7 +12955,7 @@
         <v>0.1</v>
       </c>
       <c r="J131">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K131">
         <v>10</v>
@@ -12993,7 +12993,7 @@
         <v>0.1</v>
       </c>
       <c r="J132">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K132">
         <v>10</v>
@@ -13031,7 +13031,7 @@
         <v>0.1</v>
       </c>
       <c r="J133">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K133">
         <v>10</v>
@@ -13069,7 +13069,7 @@
         <v>0.1</v>
       </c>
       <c r="J134">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K134">
         <v>10</v>
@@ -13107,7 +13107,7 @@
         <v>0.1</v>
       </c>
       <c r="J135">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K135">
         <v>10</v>
@@ -13145,7 +13145,7 @@
         <v>0.2</v>
       </c>
       <c r="J136">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K136">
         <v>10</v>
@@ -13183,7 +13183,7 @@
         <v>0.1</v>
       </c>
       <c r="J137">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K137">
         <v>10</v>
@@ -13221,7 +13221,7 @@
         <v>0.1</v>
       </c>
       <c r="J138">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K138">
         <v>10</v>
@@ -13259,7 +13259,7 @@
         <v>0.1</v>
       </c>
       <c r="J139">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K139">
         <v>10</v>
@@ -13297,7 +13297,7 @@
         <v>0.1</v>
       </c>
       <c r="J140">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K140">
         <v>10</v>
@@ -13335,7 +13335,7 @@
         <v>0.1</v>
       </c>
       <c r="J141">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K141">
         <v>10</v>
@@ -13373,7 +13373,7 @@
         <v>0.2</v>
       </c>
       <c r="J142">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K142">
         <v>10</v>
@@ -13411,7 +13411,7 @@
         <v>0.3</v>
       </c>
       <c r="J143">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K143">
         <v>8</v>
@@ -13449,7 +13449,7 @@
         <v>0.3</v>
       </c>
       <c r="J144">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K144">
         <v>14</v>
@@ -13487,7 +13487,7 @@
         <v>0.1</v>
       </c>
       <c r="J145">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K145">
         <v>10</v>
@@ -13525,7 +13525,7 @@
         <v>0.1</v>
       </c>
       <c r="J146">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K146">
         <v>9</v>
@@ -13563,7 +13563,7 @@
         <v>0.8</v>
       </c>
       <c r="J147">
-        <v>-18</v>
+        <v>0</v>
       </c>
       <c r="K147">
         <v>8</v>
@@ -13601,7 +13601,7 @@
         <v>0.17</v>
       </c>
       <c r="J148">
-        <v>-18</v>
+        <v>0</v>
       </c>
       <c r="K148">
         <v>10</v>
@@ -13639,7 +13639,7 @@
         <v>0.33</v>
       </c>
       <c r="J149">
-        <v>-18</v>
+        <v>0</v>
       </c>
       <c r="K149">
         <v>11</v>
@@ -13677,7 +13677,7 @@
         <v>0.17</v>
       </c>
       <c r="J150">
-        <v>-18</v>
+        <v>0</v>
       </c>
       <c r="K150">
         <v>10</v>
@@ -13715,7 +13715,7 @@
         <v>0.17</v>
       </c>
       <c r="J151">
-        <v>-18</v>
+        <v>0</v>
       </c>
       <c r="K151">
         <v>10</v>
@@ -13753,7 +13753,7 @@
         <v>0.17</v>
       </c>
       <c r="J152">
-        <v>-18</v>
+        <v>0</v>
       </c>
       <c r="K152">
         <v>10</v>
@@ -13791,7 +13791,7 @@
         <v>0.17</v>
       </c>
       <c r="J153">
-        <v>-18</v>
+        <v>0</v>
       </c>
       <c r="K153">
         <v>10</v>
@@ -13829,7 +13829,7 @@
         <v>0.17</v>
       </c>
       <c r="J154">
-        <v>-18</v>
+        <v>0</v>
       </c>
       <c r="K154">
         <v>10</v>
@@ -13867,7 +13867,7 @@
         <v>0.73</v>
       </c>
       <c r="J155">
-        <v>-17</v>
+        <v>0</v>
       </c>
       <c r="K155">
         <v>33</v>
@@ -13905,7 +13905,7 @@
         <v>0.4</v>
       </c>
       <c r="J156">
-        <v>-17</v>
+        <v>0</v>
       </c>
       <c r="K156">
         <v>11</v>
@@ -13943,7 +13943,7 @@
         <v>0.47</v>
       </c>
       <c r="J157">
-        <v>-17</v>
+        <v>0</v>
       </c>
       <c r="K157">
         <v>8</v>
@@ -13981,7 +13981,7 @@
         <v>0.23</v>
       </c>
       <c r="J158">
-        <v>-17</v>
+        <v>0</v>
       </c>
       <c r="K158">
         <v>10</v>
@@ -14019,7 +14019,7 @@
         <v>0.43</v>
       </c>
       <c r="J159">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="K159">
         <v>19</v>
@@ -14057,7 +14057,7 @@
         <v>0.47</v>
       </c>
       <c r="J160">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K160">
         <v>20</v>
@@ -14095,7 +14095,7 @@
         <v>0.27</v>
       </c>
       <c r="J161">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K161">
         <v>11</v>
@@ -14133,7 +14133,7 @@
         <v>0.13</v>
       </c>
       <c r="J162">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K162">
         <v>10</v>
@@ -14171,7 +14171,7 @@
         <v>0.13</v>
       </c>
       <c r="J163">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K163">
         <v>10</v>
@@ -14209,7 +14209,7 @@
         <v>0.87</v>
       </c>
       <c r="J164">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K164">
         <v>31</v>
@@ -14247,7 +14247,7 @@
         <v>0.13</v>
       </c>
       <c r="J165">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K165">
         <v>10</v>
@@ -14285,7 +14285,7 @@
         <v>0.2</v>
       </c>
       <c r="J166">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K166">
         <v>10</v>
@@ -14323,7 +14323,7 @@
         <v>0.13</v>
       </c>
       <c r="J167">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K167">
         <v>10</v>
@@ -14361,7 +14361,7 @@
         <v>0.13</v>
       </c>
       <c r="J168">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K168">
         <v>10</v>
@@ -14399,7 +14399,7 @@
         <v>0.2</v>
       </c>
       <c r="J169">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K169">
         <v>10</v>
@@ -14437,7 +14437,7 @@
         <v>0.2</v>
       </c>
       <c r="J170">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K170">
         <v>10</v>
@@ -14475,7 +14475,7 @@
         <v>0.13</v>
       </c>
       <c r="J171">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K171">
         <v>9</v>
@@ -14513,7 +14513,7 @@
         <v>0.13</v>
       </c>
       <c r="J172">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K172">
         <v>10</v>
@@ -14551,7 +14551,7 @@
         <v>0.2</v>
       </c>
       <c r="J173">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K173">
         <v>10</v>
@@ -14589,7 +14589,7 @@
         <v>0.13</v>
       </c>
       <c r="J174">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="K174">
         <v>10</v>
@@ -14627,7 +14627,7 @@
         <v>0.37</v>
       </c>
       <c r="J175">
-        <v>-13</v>
+        <v>0</v>
       </c>
       <c r="K175">
         <v>15</v>
@@ -14665,7 +14665,7 @@
         <v>0.67</v>
       </c>
       <c r="J176">
-        <v>-13</v>
+        <v>0</v>
       </c>
       <c r="K176">
         <v>14</v>
@@ -14703,7 +14703,7 @@
         <v>0.3</v>
       </c>
       <c r="J177">
-        <v>-13</v>
+        <v>0</v>
       </c>
       <c r="K177">
         <v>8</v>
@@ -14741,7 +14741,7 @@
         <v>0.53</v>
       </c>
       <c r="J178">
-        <v>-13</v>
+        <v>0</v>
       </c>
       <c r="K178">
         <v>21</v>
@@ -14779,7 +14779,7 @@
         <v>0.23</v>
       </c>
       <c r="J179">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="K179">
         <v>10</v>
@@ -14817,7 +14817,7 @@
         <v>0.7</v>
       </c>
       <c r="J180">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="K180">
         <v>13</v>
@@ -14855,7 +14855,7 @@
         <v>0.23</v>
       </c>
       <c r="J181">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="K181">
         <v>10</v>
@@ -14893,7 +14893,7 @@
         <v>0.23</v>
       </c>
       <c r="J182">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="K182">
         <v>10</v>
@@ -14931,7 +14931,7 @@
         <v>0.57</v>
       </c>
       <c r="J183">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="K183">
         <v>22</v>
@@ -14969,7 +14969,7 @@
         <v>1.47</v>
       </c>
       <c r="J184">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="K184">
         <v>14</v>
@@ -15007,7 +15007,7 @@
         <v>0.17</v>
       </c>
       <c r="J185">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="K185">
         <v>10</v>
@@ -15045,7 +15045,7 @@
         <v>0.17</v>
       </c>
       <c r="J186">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="K186">
         <v>10</v>
@@ -15083,7 +15083,7 @@
         <v>0.17</v>
       </c>
       <c r="J187">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="K187">
         <v>10</v>
@@ -15121,7 +15121,7 @@
         <v>0.17</v>
       </c>
       <c r="J188">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="K188">
         <v>10</v>
@@ -15159,7 +15159,7 @@
         <v>0.17</v>
       </c>
       <c r="J189">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="K189">
         <v>10</v>
@@ -15197,7 +15197,7 @@
         <v>0.17</v>
       </c>
       <c r="J190">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="K190">
         <v>10</v>
@@ -15235,7 +15235,7 @@
         <v>1.1</v>
       </c>
       <c r="J191">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="K191">
         <v>36</v>
@@ -15273,7 +15273,7 @@
         <v>0.43</v>
       </c>
       <c r="J192">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="K192">
         <v>11</v>
@@ -15311,7 +15311,7 @@
         <v>0.87</v>
       </c>
       <c r="J193">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="K193">
         <v>34</v>
@@ -15349,7 +15349,7 @@
         <v>0.27</v>
       </c>
       <c r="J194">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="K194">
         <v>10</v>
@@ -15387,7 +15387,7 @@
         <v>0.27</v>
       </c>
       <c r="J195">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="K195">
         <v>10</v>
@@ -15425,7 +15425,7 @@
         <v>0.57</v>
       </c>
       <c r="J196">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K196">
         <v>10</v>
@@ -15463,7 +15463,7 @@
         <v>0.57</v>
       </c>
       <c r="J197">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K197">
         <v>19</v>
@@ -15501,7 +15501,7 @@
         <v>0.1</v>
       </c>
       <c r="J198">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K198">
         <v>8</v>
@@ -15539,7 +15539,7 @@
         <v>0.1</v>
       </c>
       <c r="J199">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K199">
         <v>10</v>
@@ -15577,7 +15577,7 @@
         <v>0.1</v>
       </c>
       <c r="J200">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K200">
         <v>8</v>
@@ -15615,7 +15615,7 @@
         <v>0.1</v>
       </c>
       <c r="J201">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K201">
         <v>10</v>
@@ -15653,7 +15653,7 @@
         <v>0.1</v>
       </c>
       <c r="J202">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K202">
         <v>10</v>
@@ -15691,7 +15691,7 @@
         <v>0.1</v>
       </c>
       <c r="J203">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K203">
         <v>10</v>
@@ -15729,7 +15729,7 @@
         <v>0.2</v>
       </c>
       <c r="J204">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K204">
         <v>10</v>
@@ -15767,7 +15767,7 @@
         <v>0.1</v>
       </c>
       <c r="J205">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K205">
         <v>10</v>
@@ -15805,7 +15805,7 @@
         <v>0.4</v>
       </c>
       <c r="J206">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K206">
         <v>10</v>
@@ -15843,7 +15843,7 @@
         <v>0.1</v>
       </c>
       <c r="J207">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K207">
         <v>10</v>
@@ -15881,7 +15881,7 @@
         <v>0.3</v>
       </c>
       <c r="J208">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K208">
         <v>11</v>
@@ -15919,7 +15919,7 @@
         <v>0.6</v>
       </c>
       <c r="J209">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K209">
         <v>11</v>
@@ -15957,7 +15957,7 @@
         <v>0.1</v>
       </c>
       <c r="J210">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K210">
         <v>8</v>
@@ -15995,7 +15995,7 @@
         <v>0.1</v>
       </c>
       <c r="J211">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K211">
         <v>10</v>
@@ -16033,7 +16033,7 @@
         <v>0.1</v>
       </c>
       <c r="J212">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K212">
         <v>10</v>
@@ -16071,7 +16071,7 @@
         <v>0.1</v>
       </c>
       <c r="J213">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K213">
         <v>10</v>
@@ -16109,7 +16109,7 @@
         <v>0.1</v>
       </c>
       <c r="J214">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K214">
         <v>10</v>
@@ -16147,7 +16147,7 @@
         <v>0.1</v>
       </c>
       <c r="J215">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K215">
         <v>10</v>
@@ -16185,7 +16185,7 @@
         <v>0.2</v>
       </c>
       <c r="J216">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K216">
         <v>10</v>
@@ -16223,7 +16223,7 @@
         <v>0.1</v>
       </c>
       <c r="J217">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K217">
         <v>10</v>
@@ -16261,7 +16261,7 @@
         <v>0.1</v>
       </c>
       <c r="J218">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K218">
         <v>10</v>
@@ -16299,7 +16299,7 @@
         <v>0.1</v>
       </c>
       <c r="J219">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K219">
         <v>10</v>
@@ -16337,7 +16337,7 @@
         <v>0.1</v>
       </c>
       <c r="J220">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K220">
         <v>10</v>
@@ -16375,7 +16375,7 @@
         <v>0.1</v>
       </c>
       <c r="J221">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K221">
         <v>10</v>
@@ -16413,7 +16413,7 @@
         <v>0.1</v>
       </c>
       <c r="J222">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K222">
         <v>10</v>
@@ -16451,7 +16451,7 @@
         <v>0.1</v>
       </c>
       <c r="J223">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K223">
         <v>10</v>
@@ -16489,7 +16489,7 @@
         <v>0.1</v>
       </c>
       <c r="J224">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K224">
         <v>10</v>
@@ -16527,7 +16527,7 @@
         <v>0.1</v>
       </c>
       <c r="J225">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K225">
         <v>10</v>
@@ -16565,7 +16565,7 @@
         <v>0.1</v>
       </c>
       <c r="J226">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K226">
         <v>10</v>
@@ -16603,7 +16603,7 @@
         <v>0.1</v>
       </c>
       <c r="J227">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K227">
         <v>10</v>
@@ -16641,7 +16641,7 @@
         <v>0.1</v>
       </c>
       <c r="J228">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K228">
         <v>10</v>
@@ -16679,7 +16679,7 @@
         <v>0.3</v>
       </c>
       <c r="J229">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K229">
         <v>11</v>
@@ -16717,7 +16717,7 @@
         <v>0.1</v>
       </c>
       <c r="J230">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K230">
         <v>10</v>
@@ -16755,7 +16755,7 @@
         <v>0.43</v>
       </c>
       <c r="J231">
-        <v>-9</v>
+        <v>0</v>
       </c>
       <c r="K231">
         <v>16</v>
@@ -16793,7 +16793,7 @@
         <v>0.43</v>
       </c>
       <c r="J232">
-        <v>-9</v>
+        <v>0</v>
       </c>
       <c r="K232">
         <v>16</v>
@@ -16831,7 +16831,7 @@
         <v>0.33</v>
       </c>
       <c r="J233">
-        <v>-9</v>
+        <v>0</v>
       </c>
       <c r="K233">
         <v>12</v>
@@ -16869,7 +16869,7 @@
         <v>0.23</v>
       </c>
       <c r="J234">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="K234">
         <v>10</v>
@@ -16907,7 +16907,7 @@
         <v>0.23</v>
       </c>
       <c r="J235">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="K235">
         <v>10</v>
@@ -16945,7 +16945,7 @@
         <v>0.23</v>
       </c>
       <c r="J236">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="K236">
         <v>10</v>
@@ -16983,7 +16983,7 @@
         <v>0.23</v>
       </c>
       <c r="J237">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="K237">
         <v>10</v>
@@ -17021,7 +17021,7 @@
         <v>0.23</v>
       </c>
       <c r="J238">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="K238">
         <v>10</v>
@@ -17059,7 +17059,7 @@
         <v>0.37</v>
       </c>
       <c r="J239">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="K239">
         <v>13</v>
@@ -17097,7 +17097,7 @@
         <v>1</v>
       </c>
       <c r="J240">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="K240">
         <v>16</v>
@@ -17135,7 +17135,7 @@
         <v>1.03</v>
       </c>
       <c r="J241">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K241">
         <v>36</v>
@@ -17173,7 +17173,7 @@
         <v>0.13</v>
       </c>
       <c r="J242">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K242">
         <v>10</v>
@@ -17211,7 +17211,7 @@
         <v>0.13</v>
       </c>
       <c r="J243">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K243">
         <v>10</v>
@@ -17249,7 +17249,7 @@
         <v>0.4</v>
       </c>
       <c r="J244">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K244">
         <v>14</v>
@@ -17287,7 +17287,7 @@
         <v>0.13</v>
       </c>
       <c r="J245">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K245">
         <v>10</v>
@@ -17325,7 +17325,7 @@
         <v>0.13</v>
       </c>
       <c r="J246">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K246">
         <v>10</v>
@@ -17363,7 +17363,7 @@
         <v>0.13</v>
       </c>
       <c r="J247">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K247">
         <v>10</v>
@@ -17401,7 +17401,7 @@
         <v>0.27</v>
       </c>
       <c r="J248">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K248">
         <v>10</v>
@@ -17439,7 +17439,7 @@
         <v>0.13</v>
       </c>
       <c r="J249">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K249">
         <v>10</v>
@@ -17477,7 +17477,7 @@
         <v>0.4</v>
       </c>
       <c r="J250">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K250">
         <v>14</v>
@@ -17515,7 +17515,7 @@
         <v>0.13</v>
       </c>
       <c r="J251">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K251">
         <v>10</v>
@@ -17553,7 +17553,7 @@
         <v>0.4</v>
       </c>
       <c r="J252">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K252">
         <v>14</v>
@@ -17591,7 +17591,7 @@
         <v>0.13</v>
       </c>
       <c r="J253">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K253">
         <v>10</v>
@@ -17629,7 +17629,7 @@
         <v>0.13</v>
       </c>
       <c r="J254">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K254">
         <v>10</v>
@@ -17667,7 +17667,7 @@
         <v>0.13</v>
       </c>
       <c r="J255">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K255">
         <v>10</v>
@@ -17705,7 +17705,7 @@
         <v>0.13</v>
       </c>
       <c r="J256">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K256">
         <v>9</v>
@@ -17743,7 +17743,7 @@
         <v>0.13</v>
       </c>
       <c r="J257">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K257">
         <v>10</v>
@@ -17781,7 +17781,7 @@
         <v>0.13</v>
       </c>
       <c r="J258">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K258">
         <v>9</v>
@@ -17819,7 +17819,7 @@
         <v>0.13</v>
       </c>
       <c r="J259">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K259">
         <v>10</v>
@@ -17857,7 +17857,7 @@
         <v>0.13</v>
       </c>
       <c r="J260">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K260">
         <v>10</v>
@@ -17895,7 +17895,7 @@
         <v>0.13</v>
       </c>
       <c r="J261">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K261">
         <v>10</v>
@@ -17933,7 +17933,7 @@
         <v>0.4</v>
       </c>
       <c r="J262">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K262">
         <v>10</v>
@@ -17971,7 +17971,7 @@
         <v>0.13</v>
       </c>
       <c r="J263">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K263">
         <v>10</v>
@@ -18009,7 +18009,7 @@
         <v>0.13</v>
       </c>
       <c r="J264">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K264">
         <v>10</v>
@@ -18047,7 +18047,7 @@
         <v>0.7</v>
       </c>
       <c r="J265">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K265">
         <v>15</v>
@@ -18085,7 +18085,7 @@
         <v>0.3</v>
       </c>
       <c r="J266">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K266">
         <v>10</v>
@@ -18123,7 +18123,7 @@
         <v>0.3</v>
       </c>
       <c r="J267">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K267">
         <v>10</v>
@@ -18161,7 +18161,7 @@
         <v>1.27</v>
       </c>
       <c r="J268">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K268">
         <v>43</v>
@@ -18199,7 +18199,7 @@
         <v>0.17</v>
       </c>
       <c r="J269">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K269">
         <v>10</v>
@@ -18237,7 +18237,7 @@
         <v>0.5</v>
       </c>
       <c r="J270">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K270">
         <v>17</v>
@@ -18275,7 +18275,7 @@
         <v>0.17</v>
       </c>
       <c r="J271">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K271">
         <v>10</v>
@@ -18313,7 +18313,7 @@
         <v>0.17</v>
       </c>
       <c r="J272">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K272">
         <v>10</v>
@@ -18351,7 +18351,7 @@
         <v>0.33</v>
       </c>
       <c r="J273">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K273">
         <v>11</v>
@@ -18389,7 +18389,7 @@
         <v>0.33</v>
       </c>
       <c r="J274">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K274">
         <v>11</v>
@@ -18427,7 +18427,7 @@
         <v>0.17</v>
       </c>
       <c r="J275">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K275">
         <v>10</v>
@@ -18465,7 +18465,7 @@
         <v>0.17</v>
       </c>
       <c r="J276">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K276">
         <v>10</v>
@@ -18503,7 +18503,7 @@
         <v>0.17</v>
       </c>
       <c r="J277">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K277">
         <v>10</v>
@@ -18541,7 +18541,7 @@
         <v>0.17</v>
       </c>
       <c r="J278">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K278">
         <v>10</v>
@@ -18579,7 +18579,7 @@
         <v>0.5</v>
       </c>
       <c r="J279">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K279">
         <v>16</v>
@@ -18617,7 +18617,7 @@
         <v>0.17</v>
       </c>
       <c r="J280">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K280">
         <v>10</v>
@@ -18655,7 +18655,7 @@
         <v>0.17</v>
       </c>
       <c r="J281">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K281">
         <v>10</v>
@@ -18693,7 +18693,7 @@
         <v>0.17</v>
       </c>
       <c r="J282">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K282">
         <v>10</v>
@@ -18731,7 +18731,7 @@
         <v>0.17</v>
       </c>
       <c r="J283">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K283">
         <v>10</v>
@@ -18769,7 +18769,7 @@
         <v>0.17</v>
       </c>
       <c r="J284">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K284">
         <v>8</v>
@@ -18807,7 +18807,7 @@
         <v>0.17</v>
       </c>
       <c r="J285">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="K285">
         <v>10</v>
@@ -18845,7 +18845,7 @@
         <v>0.93</v>
       </c>
       <c r="J286">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="K286">
         <v>31</v>
@@ -18883,7 +18883,7 @@
         <v>0.4</v>
       </c>
       <c r="J287">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="K287">
         <v>13</v>
@@ -18921,7 +18921,7 @@
         <v>0.8</v>
       </c>
       <c r="J288">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="K288">
         <v>26</v>
@@ -18959,7 +18959,7 @@
         <v>0.2</v>
       </c>
       <c r="J289">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="K289">
         <v>10</v>
@@ -18997,7 +18997,7 @@
         <v>0.8</v>
       </c>
       <c r="J290">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="K290">
         <v>10</v>
@@ -19035,7 +19035,7 @@
         <v>0.4</v>
       </c>
       <c r="J291">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="K291">
         <v>13</v>
@@ -19073,7 +19073,7 @@
         <v>0.2</v>
       </c>
       <c r="J292">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="K292">
         <v>10</v>
@@ -19111,7 +19111,7 @@
         <v>0.2</v>
       </c>
       <c r="J293">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="K293">
         <v>10</v>
@@ -19149,7 +19149,7 @@
         <v>0.2</v>
       </c>
       <c r="J294">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="K294">
         <v>10</v>
@@ -19187,7 +19187,7 @@
         <v>0.2</v>
       </c>
       <c r="J295">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="K295">
         <v>10</v>
@@ -19225,7 +19225,7 @@
         <v>0.2</v>
       </c>
       <c r="J296">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="K296">
         <v>8</v>
@@ -19263,7 +19263,7 @@
         <v>0.4</v>
       </c>
       <c r="J297">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="K297">
         <v>13</v>
@@ -19301,7 +19301,7 @@
         <v>1.07</v>
       </c>
       <c r="J298">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="K298">
         <v>34</v>
@@ -19339,7 +19339,7 @@
         <v>0.43</v>
       </c>
       <c r="J299">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="K299">
         <v>14</v>
@@ -19377,7 +19377,7 @@
         <v>0.23</v>
       </c>
       <c r="J300">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="K300">
         <v>10</v>
@@ -19415,7 +19415,7 @@
         <v>0.23</v>
       </c>
       <c r="J301">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="K301">
         <v>10</v>
@@ -19453,7 +19453,7 @@
         <v>0.23</v>
       </c>
       <c r="J302">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="K302">
         <v>10</v>
@@ -19491,7 +19491,7 @@
         <v>0.23</v>
       </c>
       <c r="J303">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="K303">
         <v>10</v>
@@ -19529,7 +19529,7 @@
         <v>0.23</v>
       </c>
       <c r="J304">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="K304">
         <v>10</v>
@@ -19567,7 +19567,7 @@
         <v>0.23</v>
       </c>
       <c r="J305">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="K305">
         <v>10</v>
@@ -19605,7 +19605,7 @@
         <v>0.23</v>
       </c>
       <c r="J306">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="K306">
         <v>10</v>
@@ -19643,7 +19643,7 @@
         <v>0.23</v>
       </c>
       <c r="J307">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="K307">
         <v>10</v>
@@ -19681,7 +19681,7 @@
         <v>0.47</v>
       </c>
       <c r="J308">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="K308">
         <v>15</v>
@@ -19719,7 +19719,7 @@
         <v>2.77</v>
       </c>
       <c r="J309">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K309">
         <v>88</v>
@@ -19757,7 +19757,7 @@
         <v>0.27</v>
       </c>
       <c r="J310">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K310">
         <v>10</v>
@@ -19795,7 +19795,7 @@
         <v>0.27</v>
       </c>
       <c r="J311">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K311">
         <v>10</v>
@@ -19833,7 +19833,7 @@
         <v>0.27</v>
       </c>
       <c r="J312">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K312">
         <v>10</v>
@@ -19871,7 +19871,7 @@
         <v>0.27</v>
       </c>
       <c r="J313">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K313">
         <v>10</v>
@@ -19909,7 +19909,7 @@
         <v>0.57</v>
       </c>
       <c r="J314">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K314">
         <v>17</v>
@@ -19947,7 +19947,7 @@
         <v>0.3</v>
       </c>
       <c r="J315">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K315">
         <v>8</v>
@@ -19985,7 +19985,7 @@
         <v>0.3</v>
       </c>
       <c r="J316">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K316">
         <v>10</v>
@@ -20023,7 +20023,7 @@
         <v>0.3</v>
       </c>
       <c r="J317">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K317">
         <v>10</v>
@@ -20061,7 +20061,7 @@
         <v>3.33</v>
       </c>
       <c r="J318">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K318">
         <v>21</v>
@@ -20099,7 +20099,7 @@
         <v>0.33</v>
       </c>
       <c r="J319">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K319">
         <v>10</v>
@@ -20137,7 +20137,7 @@
         <v>0.33</v>
       </c>
       <c r="J320">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K320">
         <v>10</v>
@@ -20175,7 +20175,7 @@
         <v>0.33</v>
       </c>
       <c r="J321">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K321">
         <v>10</v>
@@ -20213,7 +20213,7 @@
         <v>0.33</v>
       </c>
       <c r="J322">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="K322">
         <v>10</v>
@@ -20251,7 +20251,7 @@
         <v>0.7</v>
       </c>
       <c r="J323">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K323">
         <v>21</v>
@@ -20289,7 +20289,7 @@
         <v>0.7</v>
       </c>
       <c r="J324">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K324">
         <v>21</v>
@@ -20327,7 +20327,7 @@
         <v>0.37</v>
       </c>
       <c r="J325">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K325">
         <v>8</v>
@@ -20365,7 +20365,7 @@
         <v>0.37</v>
       </c>
       <c r="J326">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K326">
         <v>11</v>
@@ -20403,7 +20403,7 @@
         <v>0.37</v>
       </c>
       <c r="J327">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K327">
         <v>11</v>
@@ -20441,7 +20441,7 @@
         <v>0.4</v>
       </c>
       <c r="J328">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K328">
         <v>12</v>
@@ -20479,7 +20479,7 @@
         <v>0.4</v>
       </c>
       <c r="J329">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K329">
         <v>12</v>
@@ -20517,7 +20517,7 @@
         <v>0.4</v>
       </c>
       <c r="J330">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K330">
         <v>12</v>
@@ -20555,7 +20555,7 @@
         <v>0.4</v>
       </c>
       <c r="J331">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K331">
         <v>12</v>
@@ -20593,7 +20593,7 @@
         <v>0.4</v>
       </c>
       <c r="J332">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K332">
         <v>12</v>
@@ -20631,7 +20631,7 @@
         <v>0.4</v>
       </c>
       <c r="J333">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K333">
         <v>12</v>
@@ -20669,7 +20669,7 @@
         <v>0.4</v>
       </c>
       <c r="J334">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K334">
         <v>12</v>
@@ -20707,7 +20707,7 @@
         <v>0.43</v>
       </c>
       <c r="J335">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K335">
         <v>13</v>
@@ -20745,7 +20745,7 @@
         <v>0.43</v>
       </c>
       <c r="J336">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K336">
         <v>13</v>
@@ -20783,7 +20783,7 @@
         <v>0.43</v>
       </c>
       <c r="J337">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K337">
         <v>13</v>
@@ -20821,7 +20821,7 @@
         <v>0.93</v>
       </c>
       <c r="J338">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K338">
         <v>28</v>
@@ -20859,7 +20859,7 @@
         <v>0.97</v>
       </c>
       <c r="J339">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K339">
         <v>29</v>
@@ -20897,7 +20897,7 @@
         <v>0.5</v>
       </c>
       <c r="J340">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K340">
         <v>15</v>
@@ -20935,7 +20935,7 @@
         <v>0.5</v>
       </c>
       <c r="J341">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="K341">
         <v>15</v>
@@ -20973,7 +20973,7 @@
         <v>0.53</v>
       </c>
       <c r="J342">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K342">
         <v>15</v>
@@ -21011,7 +21011,7 @@
         <v>0.53</v>
       </c>
       <c r="J343">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K343">
         <v>15</v>
@@ -21049,7 +21049,7 @@
         <v>0.53</v>
       </c>
       <c r="J344">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K344">
         <v>15</v>
@@ -21087,7 +21087,7 @@
         <v>0.6</v>
       </c>
       <c r="J345">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K345">
         <v>17</v>
@@ -21125,7 +21125,7 @@
         <v>0.63</v>
       </c>
       <c r="J346">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K346">
         <v>18</v>
@@ -21163,7 +21163,7 @@
         <v>0.67</v>
       </c>
       <c r="J347">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K347">
         <v>19</v>
@@ -21201,7 +21201,7 @@
         <v>0.67</v>
       </c>
       <c r="J348">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K348">
         <v>16</v>
@@ -21239,7 +21239,7 @@
         <v>1.5</v>
       </c>
       <c r="J349">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K349">
         <v>20</v>
@@ -21277,7 +21277,7 @@
         <v>0.8</v>
       </c>
       <c r="J350">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K350">
         <v>23</v>
@@ -21315,7 +21315,7 @@
         <v>0.9</v>
       </c>
       <c r="J351">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K351">
         <v>9</v>

</xml_diff>